<commit_message>
feat(voucher): phan tich URD docx + gen TC UI man hinh Thanh toan
- Phan tich DOC-VOUCHER-07/08 (.docx ban goc): extract anh UI thuc te
  → bo sung MODULE VOUCHER-AUTO-UI (6 SC) + VOUCHER-UI (12 SC)
  → them CLA-VOUCHER-007/008, CLA-AUTO-001/002/003
- Gen TC Web UI: AI_ISC_ecom-pdh_v1.1_TC_v1.0.xlsx (18 TC, 6 nhom)
  High:12 | Medium:6 | BLOCKED:2 (CLA-AUTO-001, CLA-AUTO-003)
- Cap nhat TC API: v1.0 -> v1.1 (100 TC, fix Content1-6 spec)
- Cap nhat MEMORY.md, requirement_traceability.md, test_scenario_map.md
- Cap nhat CLAUDE.md: 60 REQ / 63 SC / 9 modules / 15 CLAs

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ecom-pdh/00_input/chucnang_Voucher/api doc v1.xlsx
+++ b/ecom-pdh/00_input/chucnang_Voucher/api doc v1.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\AI\Ecom\ecom-pdh\00_input\chucnang_Voucher\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12390" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12390" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Rule chung cho header" sheetId="5" r:id="rId1"/>
@@ -22,18 +22,86 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
+  <si>
+    <t>X-Checkout-Token</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bắt buộc </t>
+  </si>
+  <si>
+    <t>Client-Id</t>
+  </si>
+  <si>
+    <t>Không băt buộc</t>
+  </si>
+  <si>
+    <t>Authorization</t>
+  </si>
+  <si>
+    <t>Không nhập báo lỗi cho người dùng, không hiển thị voucher
+Nhập sai báo lỗi không lấy được voucher
+Hết hạn báo lỗi, không hiển thị voucher</t>
+  </si>
+  <si>
+    <t>Trường hợp có data thông tin body trả ra mỗi voucher có đủ các thành phần theo BA yêu cầu 
+Mã EVC. ⚠ Client cần lưu lại để dùng khi apply.
+Mô tả nội dung khuyến mãi. 
+Ghi chú (có thể rỗng). Mapping: Note
+Ngày hết hạn voucher, format dd/MM/yyyy. 
+Loại EVC. ⚠ Client phải lưu lại — bắt buộc truyền vào khi apply. 
+Hình thức áp dụng EVC.
+Loại khuyến mãi.
+Nhóm chính sách.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trường hợp có data thông tin body trả ra  có đủ các thành phần theo BA yêu cầu: 
+ID promotion
+Tiêu đề promotion
+Mã voucher
+referrer_code
+Loại giảm giá
+Giá trị giảm giá
+Giá trị giảm giá chưa VAT
+% giảm giá
+Hình thức áp dụng
+Giá trị giảm giá gốc
+Giá trị giảm giá gốc chưa VAT
+voucher_type
+voucher_type_l2
+type_id
+Sản phẩm áp dụng
+service _id
+discount_ex_vat 
+discount 
+dismonth 
+is_deduct_order 
+original_discount_value 
+original_discount_ex_vat 
+</t>
+  </si>
+  <si>
+    <t>Trường hợp có data thông tin body trả ra  có đủ các thành phần theo BA yêu cầu: 
+Mã voucher
+Content1
+Content2
+Content3
+Content4
+Content5
+Content6</t>
+  </si>
   <si>
     <t>curl --location --request POST '/public/v1/voucher/list' \
 --header 'X-Checkout-Token;' \
---header 'Accept-Language;' \
 --header 'Client-Id;' \
 --header 'Authorization: Bearer &lt;token&gt;'</t>
   </si>
   <si>
     <t>curl --location '/public/v1/voucher/content' \
 --header 'X-Checkout-Token;' \
---header 'Accept-Language;' \
 --header 'Client-Id;' \
 --header 'Authorization: Bearer &lt;token&gt;' \
 --header 'Content-Type: application/json' \
@@ -44,7 +112,6 @@
   <si>
     <t>curl --location '/public/v1/voucher/apply' \
 --header 'X-Checkout-Token;' \
---header 'Accept-Language;' \
 --header 'Client-Id;' \
 --header 'Authorization: Bearer &lt;token&gt;' \
 --header 'Content-Type: application/json' \
@@ -60,69 +127,6 @@
         }
     ]
 }'</t>
-  </si>
-  <si>
-    <t>X-Checkout-Token</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bắt buộc </t>
-  </si>
-  <si>
-    <t>Client-Id</t>
-  </si>
-  <si>
-    <t>Không băt buộc</t>
-  </si>
-  <si>
-    <t>Authorization</t>
-  </si>
-  <si>
-    <t>Không nhập báo lỗi cho người dùng, không hiển thị voucher
-Nhập sai báo lỗi không lấy được voucher
-Hết hạn báo lỗi, không hiển thị voucher</t>
-  </si>
-  <si>
-    <t>Trường hợp có data thông tin body trả ra  có đủ các thành phần theo BA yêu cầu: 
-Mã promotion
-Tiêu đề chương trình khuyến mãi
-Mã EVC
-Mã giới thiệu
-Loại giảm giá (ví dụ: Amount)
-Tổng Giá trị giảm đã bao gồm VAT (VNĐ)
-Tổng Giá trị giảm chưa bao gồm VAT (VNĐ)
-Tỷ lệ giảm giá (%)
-Hình thức áp dụng (ví dụ: immediate)
-Thời điểm bắt đầu áp dụng
-Thời điểm kết thúc áp dụng
-Tổng Giá trị giảm gốc đã VAT
-Tổng Giá trị giảm gốc chưa VAT
-Loại EVC cấp 1
-Loại EVC cấp 2
-ID loại voucher
-ID dịch vụ được áp chiết khấu
-ID loại sub-service
-ID sub-service cụ thể
-Mã dịch vụ
-Tiền giảm chưa VAT
-Tiền giảm đã VAT
-Số tháng giảm (0 = áp 1 lần)
-1 = khấu trừ thẳng vào tổng đơn
-Giá trị giảm gốc đã VAT theo dịch vụ
-Giá trị giảm gốc chưa VAT theo dịch vụ</t>
-  </si>
-  <si>
-    <t>Trường hợp có data thông tin body trả ra mỗi voucher có đủ các thành phần theo BA yêu cầu 
-Mã EVC. ⚠ Client cần lưu lại để dùng khi apply.
-Mô tả nội dung khuyến mãi. 
-Ghi chú (có thể rỗng). Mapping: Note
-Ngày hết hạn voucher, format dd/MM/yyyy. 
-Loại EVC. ⚠ Client phải lưu lại — bắt buộc truyền vào khi apply. 
-Hình thức áp dụng EVC.
-Loại khuyến mãi.
-Nhóm chính sách.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -513,32 +517,32 @@
   <sheetData>
     <row r="5" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B5" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -569,10 +573,10 @@
   <sheetData>
     <row r="1" spans="1:11" ht="150" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="8"/>
@@ -623,9 +627,9 @@
     <col min="11" max="11" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="135" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>9</v>
@@ -678,15 +682,15 @@
     <col min="11" max="11" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="405" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="360" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C1" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="8"/>

</xml_diff>